<commit_message>
FIX: Fixes from PR
</commit_message>
<xml_diff>
--- a/xlsx/tests/calc_tests/ADDRESS.xlsx
+++ b/xlsx/tests/calc_tests/ADDRESS.xlsx
@@ -8,14 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nhatcher/Documents/Excel/LOOKUP_AND_REFERENCE/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB98C902-E6AF-0543-AA55-1D9B56DBBA1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7ADE71F3-0944-314D-B154-E7B45003501A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16800" yWindow="640" windowWidth="16820" windowHeight="18580" xr2:uid="{870501CD-A160-5F42-938F-16F65ECEC4C0}"/>
+    <workbookView xWindow="16780" yWindow="620" windowWidth="16820" windowHeight="18580" xr2:uid="{870501CD-A160-5F42-938F-16F65ECEC4C0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="A Wird One$" sheetId="3" r:id="rId2"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -447,14 +449,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA01282A-8EE0-C644-B00B-04464CC96FCE}">
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G40"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="5" max="5" width="29.1640625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="E2" t="str">
+        <f>ADDRESS(2,3,1,1,"Sheet2")</f>
+        <v>Sheet2!$C$2</v>
+      </c>
+    </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="C5" t="str">
         <f>ADDRESS(1,1)</f>
@@ -707,7 +718,55 @@
         <v>#VALUE!</v>
       </c>
     </row>
+    <row r="33" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B33" t="str">
+        <f>ADDRESS(1,1,1,1,"A Wird One$")</f>
+        <v>'A Wird One$'!$A$1</v>
+      </c>
+    </row>
+    <row r="35" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B35" cm="1">
+        <f t="array" aca="1" ref="B35" ca="1">INDIRECT(B33)</f>
+        <v>23</v>
+      </c>
+    </row>
+    <row r="38" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B38" t="str">
+        <f>ADDRESS(2,3,1,1,"Me lo invente")</f>
+        <v>'Me lo invente'!$C$2</v>
+      </c>
+    </row>
+    <row r="40" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B40" t="e">
+        <f>ADDRESS(2,3,5)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D8A0543-C96B-714C-86F4-1350C85BD384}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1">
+        <v>23</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D3BC6DB-9F29-3F44-9ACE-3FA7BA01EDBF}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>